<commit_message>
Mark direct household enrolment delivery complete
</commit_message>
<xml_diff>
--- a/docs/08_sprint_plan.xlsx
+++ b/docs/08_sprint_plan.xlsx
@@ -1561,7 +1561,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1574,7 +1574,6 @@
           <t>Current delivery</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
           <t>Direct household enrolment — Beneficiaries selection panel, canonical Programme + effective DSA + saved geography validation, atomic ProgrammeEnrolment batch, audit and cross-view SSOT checks.</t>
@@ -4267,12 +4266,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>(working tree)</t>
+          <t>df576fe</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -9317,7 +9316,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">

</xml_diff>